<commit_message>
France daily ratings for 2026-03-23
</commit_message>
<xml_diff>
--- a/output/daily_ratings/france_ratings_2026-03-23.xlsx
+++ b/output/daily_ratings/france_ratings_2026-03-23.xlsx
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>85.02004813388832</v>
+        <v>65.96756728225006</v>
       </c>
       <c r="T2" t="n">
-        <v>85.02004813388832</v>
+        <v>65.96756728225006</v>
       </c>
     </row>
     <row r="3">
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>89.23106659765109</v>
+        <v>70.05652783303222</v>
       </c>
       <c r="T3" t="n">
-        <v>89.23106659765109</v>
+        <v>70.05652783303222</v>
       </c>
     </row>
     <row r="4">
@@ -736,10 +736,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>78.68414566387486</v>
+        <v>59.815313266641</v>
       </c>
       <c r="T4" t="n">
-        <v>78.68414566387486</v>
+        <v>59.815313266641</v>
       </c>
     </row>
     <row r="5">
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>71.45207495662871</v>
+        <v>52.79286677848835</v>
       </c>
       <c r="T5" t="n">
-        <v>71.45207495662871</v>
+        <v>52.79286677848835</v>
       </c>
     </row>
     <row r="6">
@@ -884,10 +884,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>73.72042370717764</v>
+        <v>54.99546660943822</v>
       </c>
       <c r="T6" t="n">
-        <v>73.72042370717764</v>
+        <v>54.99546660943822</v>
       </c>
     </row>
     <row r="7">
@@ -958,10 +958,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>78.78549108213896</v>
+        <v>59.91372115082638</v>
       </c>
       <c r="T7" t="n">
-        <v>78.78549108213896</v>
+        <v>59.91372115082638</v>
       </c>
     </row>
     <row r="8">
@@ -1032,10 +1032,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>73.22393488760278</v>
+        <v>54.51336870019941</v>
       </c>
       <c r="T8" t="n">
-        <v>73.22393488760278</v>
+        <v>54.51336870019941</v>
       </c>
     </row>
     <row r="9">
@@ -1106,10 +1106,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>73.15447052362718</v>
+        <v>54.4459177862636</v>
       </c>
       <c r="T9" t="n">
-        <v>73.15447052362718</v>
+        <v>54.4459177862636</v>
       </c>
     </row>
     <row r="10">
@@ -1180,10 +1180,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>73.85365017973027</v>
+        <v>55.12483146387316</v>
       </c>
       <c r="T10" t="n">
-        <v>73.85365017973027</v>
+        <v>55.12483146387316</v>
       </c>
     </row>
     <row r="11">
@@ -1254,10 +1254,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>74.92633045460127</v>
+        <v>56.16641970797468</v>
       </c>
       <c r="T11" t="n">
-        <v>74.92633045460127</v>
+        <v>56.16641970797468</v>
       </c>
     </row>
     <row r="12">
@@ -1328,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>73.28769699617979</v>
+        <v>54.57528264069852</v>
       </c>
       <c r="T12" t="n">
-        <v>73.28769699617979</v>
+        <v>54.57528264069852</v>
       </c>
     </row>
     <row r="13">
@@ -1402,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>64.58780261275186</v>
+        <v>46.12755788339092</v>
       </c>
       <c r="T13" t="n">
-        <v>64.58780261275186</v>
+        <v>46.12755788339092</v>
       </c>
     </row>
     <row r="14">
@@ -1476,10 +1476,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>65.83012643081102</v>
+        <v>47.33387249042826</v>
       </c>
       <c r="T14" t="n">
-        <v>65.83012643081102</v>
+        <v>47.33387249042826</v>
       </c>
     </row>
     <row r="15">
@@ -1550,10 +1550,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>54.2799895861394</v>
+        <v>36.11852059387135</v>
       </c>
       <c r="T15" t="n">
-        <v>54.2799895861394</v>
+        <v>36.11852059387135</v>
       </c>
     </row>
     <row r="16">
@@ -1624,10 +1624,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>59.56368832477315</v>
+        <v>41.24906938875502</v>
       </c>
       <c r="T16" t="n">
-        <v>59.56368832477315</v>
+        <v>41.24906938875502</v>
       </c>
     </row>
     <row r="17">
@@ -1697,13 +1697,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R17" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>83.6270825098307</v>
+        <v>55.63024521746672</v>
       </c>
       <c r="T17" t="n">
-        <v>83.6270825098307</v>
+        <v>55.63024521746672</v>
       </c>
     </row>
     <row r="18">
@@ -1771,13 +1771,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R18" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>81.9582716144958</v>
+        <v>54.00980541734232</v>
       </c>
       <c r="T18" t="n">
-        <v>81.9582716144958</v>
+        <v>54.00980541734232</v>
       </c>
     </row>
     <row r="19">
@@ -1845,13 +1845,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R19" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>80.15559070791082</v>
+        <v>52.25937587729044</v>
       </c>
       <c r="T19" t="n">
-        <v>80.15559070791082</v>
+        <v>52.25937587729044</v>
       </c>
     </row>
     <row r="20">
@@ -1919,13 +1919,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R20" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>78.35290980132581</v>
+        <v>50.50894633723854</v>
       </c>
       <c r="T20" t="n">
-        <v>78.35290980132581</v>
+        <v>50.50894633723854</v>
       </c>
     </row>
     <row r="21">
@@ -1993,13 +1993,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R21" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>74.74754798815582</v>
+        <v>47.00808725713476</v>
       </c>
       <c r="T21" t="n">
-        <v>74.74754798815582</v>
+        <v>47.00808725713476</v>
       </c>
     </row>
     <row r="22">
@@ -2067,13 +2067,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R22" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>71.74307981051417</v>
+        <v>44.09070469038161</v>
       </c>
       <c r="T22" t="n">
-        <v>71.74307981051417</v>
+        <v>44.09070469038161</v>
       </c>
     </row>
     <row r="23">
@@ -2141,13 +2141,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R23" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>68.73861163287251</v>
+        <v>41.17332212362846</v>
       </c>
       <c r="T23" t="n">
-        <v>68.73861163287251</v>
+        <v>41.17332212362846</v>
       </c>
     </row>
     <row r="24">
@@ -2217,13 +2217,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R24" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>93.72252376329538</v>
+        <v>65.43306640749073</v>
       </c>
       <c r="T24" t="n">
-        <v>93.72252376329538</v>
+        <v>65.43306640749073</v>
       </c>
     </row>
     <row r="25">
@@ -2291,13 +2291,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R25" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>90.69568311751877</v>
+        <v>62.4939598467882</v>
       </c>
       <c r="T25" t="n">
-        <v>90.69568311751877</v>
+        <v>62.4939598467882</v>
       </c>
     </row>
     <row r="26">
@@ -2365,13 +2365,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R26" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>90.09031498836345</v>
+        <v>61.9061385346477</v>
       </c>
       <c r="T26" t="n">
-        <v>90.09031498836345</v>
+        <v>61.9061385346477</v>
       </c>
     </row>
     <row r="27">
@@ -2439,13 +2439,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R27" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>82.82589743849957</v>
+        <v>54.85228278896164</v>
       </c>
       <c r="T27" t="n">
-        <v>82.82589743849957</v>
+        <v>54.85228278896164</v>
       </c>
     </row>
     <row r="28">
@@ -2513,13 +2513,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R28" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>82.46267656100638</v>
+        <v>54.49959000167733</v>
       </c>
       <c r="T28" t="n">
-        <v>82.46267656100638</v>
+        <v>54.49959000167733</v>
       </c>
     </row>
     <row r="29">
@@ -2587,13 +2587,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R29" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>79.43583591522975</v>
+        <v>51.56048344097481</v>
       </c>
       <c r="T29" t="n">
-        <v>79.43583591522975</v>
+        <v>51.56048344097481</v>
       </c>
     </row>
     <row r="30">
@@ -2661,13 +2661,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R30" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>79.19368866356763</v>
+        <v>51.32535491611861</v>
       </c>
       <c r="T30" t="n">
-        <v>79.19368866356763</v>
+        <v>51.32535491611861</v>
       </c>
     </row>
     <row r="31">
@@ -2735,13 +2735,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R31" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>78.83046778607442</v>
+        <v>50.9726621288343</v>
       </c>
       <c r="T31" t="n">
-        <v>78.83046778607442</v>
+        <v>50.9726621288343</v>
       </c>
     </row>
     <row r="32">
@@ -2809,13 +2809,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R32" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>72.66528895140605</v>
+        <v>44.98618326145113</v>
       </c>
       <c r="T32" t="n">
-        <v>72.66528895140605</v>
+        <v>44.98618326145113</v>
       </c>
     </row>
     <row r="33">
@@ -2883,13 +2883,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R33" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>70.96068210705522</v>
+        <v>43.33098507100774</v>
       </c>
       <c r="T33" t="n">
-        <v>70.96068210705522</v>
+        <v>43.33098507100774</v>
       </c>
     </row>
     <row r="34">
@@ -2957,13 +2957,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R34" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>61.27479204057006</v>
+        <v>33.92584407675966</v>
       </c>
       <c r="T34" t="n">
-        <v>61.27479204057006</v>
+        <v>33.92584407675966</v>
       </c>
     </row>
     <row r="35">
@@ -3031,13 +3031,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R35" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>54.01037449070618</v>
+        <v>26.8719883310736</v>
       </c>
       <c r="T35" t="n">
-        <v>54.01037449070618</v>
+        <v>26.8719883310736</v>
       </c>
     </row>
     <row r="36">
@@ -3107,13 +3107,13 @@
         <v>0.7656499999999937</v>
       </c>
       <c r="R36" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>67.64938058752314</v>
+        <v>40.77469380704136</v>
       </c>
       <c r="T36" t="n">
-        <v>67.64938058752314</v>
+        <v>40.77469380704136</v>
       </c>
     </row>
     <row r="37">
@@ -3181,13 +3181,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R37" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>64.34486426652337</v>
+        <v>37.56596010229521</v>
       </c>
       <c r="T37" t="n">
-        <v>64.34486426652337</v>
+        <v>37.56596010229521</v>
       </c>
     </row>
     <row r="38">
@@ -3255,13 +3255,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R38" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>64.0596354627241</v>
+        <v>37.28899875987452</v>
       </c>
       <c r="T38" t="n">
-        <v>64.0596354627241</v>
+        <v>37.28899875987452</v>
       </c>
     </row>
     <row r="39">
@@ -3329,13 +3329,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R39" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>63.58425412305863</v>
+        <v>36.8273965225067</v>
       </c>
       <c r="T39" t="n">
-        <v>63.58425412305863</v>
+        <v>36.8273965225067</v>
       </c>
     </row>
     <row r="40">
@@ -3403,13 +3403,13 @@
         <v>0.7656499999999937</v>
       </c>
       <c r="R40" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>65.65277896092815</v>
+        <v>38.83596441009649</v>
       </c>
       <c r="T40" t="n">
-        <v>65.65277896092815</v>
+        <v>38.83596441009649</v>
       </c>
     </row>
     <row r="41">
@@ -3477,13 +3477,13 @@
         <v>0.7656499999999937</v>
       </c>
       <c r="R41" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>61.84972824360436</v>
+        <v>35.14314651115391</v>
       </c>
       <c r="T41" t="n">
-        <v>61.84972824360436</v>
+        <v>35.14314651115391</v>
       </c>
     </row>
     <row r="42">
@@ -3551,13 +3551,13 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R42" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>54.28993292227387</v>
+        <v>27.80247462692599</v>
       </c>
       <c r="T42" t="n">
-        <v>54.28993292227387</v>
+        <v>27.80247462692599</v>
       </c>
     </row>
     <row r="43">
@@ -3625,13 +3625,13 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R43" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>53.33917024294292</v>
+        <v>26.87927015219035</v>
       </c>
       <c r="T43" t="n">
-        <v>53.33917024294292</v>
+        <v>26.87927015219035</v>
       </c>
     </row>
     <row r="44">
@@ -3699,13 +3699,13 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R44" t="n">
-        <v>12.04644873936213</v>
+        <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>42.88078077030245</v>
+        <v>16.72402093009823</v>
       </c>
       <c r="T44" t="n">
-        <v>42.88078077030245</v>
+        <v>16.72402093009823</v>
       </c>
     </row>
     <row r="45">
@@ -3778,10 +3778,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>82.20300502262316</v>
+        <v>63.23217719765677</v>
       </c>
       <c r="T45" t="n">
-        <v>82.20300502262316</v>
+        <v>63.23217719765677</v>
       </c>
     </row>
     <row r="46">
@@ -3852,10 +3852,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>75.65751866110017</v>
+        <v>56.87641415641971</v>
       </c>
       <c r="T46" t="n">
-        <v>75.65751866110017</v>
+        <v>56.87641415641971</v>
       </c>
     </row>
     <row r="47">
@@ -3926,10 +3926,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>80.58295141393134</v>
+        <v>61.6590814363587</v>
       </c>
       <c r="T47" t="n">
-        <v>80.58295141393134</v>
+        <v>61.6590814363587</v>
       </c>
     </row>
     <row r="48">
@@ -4000,10 +4000,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>74.99351249272416</v>
+        <v>56.23165445010881</v>
       </c>
       <c r="T48" t="n">
-        <v>74.99351249272416</v>
+        <v>56.23165445010881</v>
       </c>
     </row>
     <row r="49">
@@ -4074,10 +4074,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>72.55983522655899</v>
+        <v>53.86851821113994</v>
       </c>
       <c r="T49" t="n">
-        <v>72.55983522655899</v>
+        <v>53.86851821113994</v>
       </c>
     </row>
     <row r="50">
@@ -4148,10 +4148,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>75.02255160297457</v>
+        <v>56.25985185110943</v>
       </c>
       <c r="T50" t="n">
-        <v>75.02255160297457</v>
+        <v>56.25985185110943</v>
       </c>
     </row>
     <row r="51">
@@ -4222,10 +4222,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>67.28566886549197</v>
+        <v>48.74722549436682</v>
       </c>
       <c r="T51" t="n">
-        <v>67.28566886549197</v>
+        <v>48.74722549436682</v>
       </c>
     </row>
     <row r="52">
@@ -4296,10 +4296,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>63.95844431735708</v>
+        <v>45.51644176876879</v>
       </c>
       <c r="T52" t="n">
-        <v>63.95844431735708</v>
+        <v>45.51644176876879</v>
       </c>
     </row>
     <row r="53">
@@ -4370,10 +4370,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>72.50895071231304</v>
+        <v>53.81910860318219</v>
       </c>
       <c r="T53" t="n">
-        <v>72.50895071231304</v>
+        <v>53.81910860318219</v>
       </c>
     </row>
     <row r="54">
@@ -4444,10 +4444,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>63.71867344386801</v>
+        <v>45.28362074189365</v>
       </c>
       <c r="T54" t="n">
-        <v>63.71867344386801</v>
+        <v>45.28362074189365</v>
       </c>
     </row>
     <row r="55">
@@ -4518,10 +4518,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>57.90688711532201</v>
+        <v>39.640291169369</v>
       </c>
       <c r="T55" t="n">
-        <v>57.90688711532201</v>
+        <v>39.640291169369</v>
       </c>
     </row>
     <row r="56">
@@ -4594,10 +4594,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>92.42841574708781</v>
+        <v>73.33179361601336</v>
       </c>
       <c r="T56" t="n">
-        <v>92.42841574708781</v>
+        <v>73.33179361601336</v>
       </c>
     </row>
     <row r="57">
@@ -4668,10 +4668,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>91.56584544644329</v>
+        <v>72.4942252315565</v>
       </c>
       <c r="T57" t="n">
-        <v>91.56584544644329</v>
+        <v>72.4942252315565</v>
       </c>
     </row>
     <row r="58">
@@ -4742,10 +4742,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>86.70236665626248</v>
+        <v>67.77171615596214</v>
       </c>
       <c r="T58" t="n">
-        <v>86.70236665626248</v>
+        <v>67.77171615596214</v>
       </c>
     </row>
     <row r="59">
@@ -4816,10 +4816,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>87.84025060038609</v>
+        <v>68.87661811707402</v>
       </c>
       <c r="T59" t="n">
-        <v>87.84025060038609</v>
+        <v>68.87661811707402</v>
       </c>
     </row>
     <row r="60">
@@ -4890,10 +4890,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>84.89924030155184</v>
+        <v>66.02085407926171</v>
       </c>
       <c r="T60" t="n">
-        <v>84.89924030155184</v>
+        <v>66.02085407926171</v>
       </c>
     </row>
     <row r="61">
@@ -4964,10 +4964,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>85.37188183508842</v>
+        <v>66.47979592478508</v>
       </c>
       <c r="T61" t="n">
-        <v>85.37188183508842</v>
+        <v>66.47979592478508</v>
       </c>
     </row>
     <row r="62">
@@ -5038,10 +5038,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>81.27644503884481</v>
+        <v>62.5030668645429</v>
       </c>
       <c r="T62" t="n">
-        <v>81.27644503884481</v>
+        <v>62.5030668645429</v>
       </c>
     </row>
     <row r="63">
@@ -5112,10 +5112,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>68.92042017333529</v>
+        <v>50.50518590668864</v>
       </c>
       <c r="T63" t="n">
-        <v>68.92042017333529</v>
+        <v>50.50518590668864</v>
       </c>
     </row>
     <row r="64">
@@ -5186,10 +5186,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>76.59375158543577</v>
+        <v>57.95610299649888</v>
       </c>
       <c r="T64" t="n">
-        <v>76.59375158543577</v>
+        <v>57.95610299649888</v>
       </c>
     </row>
     <row r="65">
@@ -5260,10 +5260,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>75.65319553136965</v>
+        <v>57.04280930425533</v>
       </c>
       <c r="T65" t="n">
-        <v>75.65319553136965</v>
+        <v>57.04280930425533</v>
       </c>
     </row>
     <row r="66">
@@ -5334,10 +5334,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>71.22100189151109</v>
+        <v>52.73908442088938</v>
       </c>
       <c r="T66" t="n">
-        <v>71.22100189151109</v>
+        <v>52.73908442088938</v>
       </c>
     </row>
     <row r="67">
@@ -5408,10 +5408,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>65.29762491062827</v>
+        <v>46.98739869196982</v>
       </c>
       <c r="T67" t="n">
-        <v>65.29762491062827</v>
+        <v>46.98739869196982</v>
       </c>
     </row>
     <row r="68">
@@ -5482,10 +5482,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>65.03885382043489</v>
+        <v>46.73612817663275</v>
       </c>
       <c r="T68" t="n">
-        <v>65.03885382043489</v>
+        <v>46.73612817663275</v>
       </c>
     </row>
     <row r="69">
@@ -5556,10 +5556,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>54.68801021270055</v>
+        <v>36.68530756315042</v>
       </c>
       <c r="T69" t="n">
-        <v>54.68801021270055</v>
+        <v>36.68530756315042</v>
       </c>
     </row>
     <row r="70">
@@ -5630,10 +5630,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>54.25672506237829</v>
+        <v>36.26652337092199</v>
       </c>
       <c r="T70" t="n">
-        <v>54.25672506237829</v>
+        <v>36.26652337092199</v>
       </c>
     </row>
     <row r="71">
@@ -5706,10 +5706,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>87.66709089935799</v>
+        <v>68.74393705354575</v>
       </c>
       <c r="T71" t="n">
-        <v>87.66709089935799</v>
+        <v>68.74393705354575</v>
       </c>
     </row>
     <row r="72">
@@ -5780,10 +5780,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>83.84783115762782</v>
+        <v>65.03537995470779</v>
       </c>
       <c r="T72" t="n">
-        <v>83.84783115762782</v>
+        <v>65.03537995470779</v>
       </c>
     </row>
     <row r="73">
@@ -5854,10 +5854,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>88.33032937623702</v>
+        <v>69.387951320179</v>
       </c>
       <c r="T73" t="n">
-        <v>88.33032937623702</v>
+        <v>69.387951320179</v>
       </c>
     </row>
     <row r="74">
@@ -5928,10 +5928,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>82.60143976364176</v>
+        <v>63.82511567192203</v>
       </c>
       <c r="T74" t="n">
-        <v>82.60143976364176</v>
+        <v>63.82511567192203</v>
       </c>
     </row>
     <row r="75">
@@ -6002,10 +6002,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>85.0588563996951</v>
+        <v>66.21130318644536</v>
       </c>
       <c r="T75" t="n">
-        <v>85.0588563996951</v>
+        <v>66.21130318644536</v>
       </c>
     </row>
     <row r="76">
@@ -6076,10 +6076,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>78.66378113089424</v>
+        <v>60.00159151730116</v>
       </c>
       <c r="T76" t="n">
-        <v>78.66378113089424</v>
+        <v>60.00159151730116</v>
       </c>
     </row>
     <row r="77">
@@ -6150,10 +6150,10 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>75.74750482740434</v>
+        <v>57.16984455091626</v>
       </c>
       <c r="T77" t="n">
-        <v>75.74750482740434</v>
+        <v>57.16984455091626</v>
       </c>
     </row>
     <row r="78">
@@ -6224,10 +6224,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>74.05993684194114</v>
+        <v>55.53119134179303</v>
       </c>
       <c r="T78" t="n">
-        <v>74.05993684194114</v>
+        <v>55.53119134179303</v>
       </c>
     </row>
     <row r="79">
@@ -6298,10 +6298,10 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>72.37236885647791</v>
+        <v>53.89253813266979</v>
       </c>
       <c r="T79" t="n">
-        <v>72.37236885647791</v>
+        <v>53.89253813266979</v>
       </c>
     </row>
     <row r="80">
@@ -6372,10 +6372,10 @@
         <v>0</v>
       </c>
       <c r="S80" t="n">
-        <v>79.32112524912014</v>
+        <v>60.63988227542637</v>
       </c>
       <c r="T80" t="n">
-        <v>79.32112524912014</v>
+        <v>60.63988227542637</v>
       </c>
     </row>
     <row r="81">
@@ -6448,10 +6448,10 @@
         <v>0</v>
       </c>
       <c r="S81" t="n">
-        <v>93.8567416884177</v>
+        <v>74.82821057583487</v>
       </c>
       <c r="T81" t="n">
-        <v>93.8567416884177</v>
+        <v>74.82821057583487</v>
       </c>
     </row>
     <row r="82">
@@ -6522,10 +6522,10 @@
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>90.9024811750993</v>
+        <v>71.95958038585978</v>
       </c>
       <c r="T82" t="n">
-        <v>90.9024811750993</v>
+        <v>71.95958038585978</v>
       </c>
     </row>
     <row r="83">
@@ -6596,10 +6596,10 @@
         <v>0</v>
       </c>
       <c r="S83" t="n">
-        <v>88.11479234021138</v>
+        <v>69.25269373318829</v>
       </c>
       <c r="T83" t="n">
-        <v>88.11479234021138</v>
+        <v>69.25269373318829</v>
       </c>
     </row>
     <row r="84">
@@ -6670,10 +6670,10 @@
         <v>0</v>
       </c>
       <c r="S84" t="n">
-        <v>86.379051567335</v>
+        <v>67.56726404254434</v>
       </c>
       <c r="T84" t="n">
-        <v>86.379051567335</v>
+        <v>67.56726404254434</v>
       </c>
     </row>
     <row r="85">
@@ -6744,10 +6744,10 @@
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>91.35392236546122</v>
+        <v>72.39793638792267</v>
       </c>
       <c r="T85" t="n">
-        <v>91.35392236546122</v>
+        <v>72.39793638792267</v>
       </c>
     </row>
     <row r="86">
@@ -6818,10 +6818,10 @@
         <v>0</v>
       </c>
       <c r="S86" t="n">
-        <v>89.70146743180008</v>
+        <v>70.79337846593052</v>
       </c>
       <c r="T86" t="n">
-        <v>89.70146743180008</v>
+        <v>70.79337846593052</v>
       </c>
     </row>
     <row r="87">
@@ -6892,10 +6892,10 @@
         <v>0</v>
       </c>
       <c r="S87" t="n">
-        <v>87.26442795091603</v>
+        <v>68.42697746726822</v>
       </c>
       <c r="T87" t="n">
-        <v>87.26442795091603</v>
+        <v>68.42697746726822</v>
       </c>
     </row>
     <row r="88">
@@ -6966,10 +6966,10 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>87.18114211170077</v>
+        <v>68.3461056986164</v>
       </c>
       <c r="T88" t="n">
-        <v>87.18114211170077</v>
+        <v>68.3461056986164</v>
       </c>
     </row>
     <row r="89">
@@ -7040,10 +7040,10 @@
         <v>0</v>
       </c>
       <c r="S89" t="n">
-        <v>87.70536554299224</v>
+        <v>68.85513432168996</v>
       </c>
       <c r="T89" t="n">
-        <v>87.70536554299224</v>
+        <v>68.85513432168996</v>
       </c>
     </row>
     <row r="90">
@@ -7114,10 +7114,10 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>80.12688358555145</v>
+        <v>61.49631744034569</v>
       </c>
       <c r="T90" t="n">
-        <v>80.12688358555145</v>
+        <v>61.49631744034569</v>
       </c>
     </row>
     <row r="91">
@@ -7188,10 +7188,10 @@
         <v>0</v>
       </c>
       <c r="S91" t="n">
-        <v>84.57402975295764</v>
+        <v>65.8145614467701</v>
       </c>
       <c r="T91" t="n">
-        <v>84.57402975295764</v>
+        <v>65.8145614467701</v>
       </c>
     </row>
     <row r="92">
@@ -7262,10 +7262,10 @@
         <v>0</v>
       </c>
       <c r="S92" t="n">
-        <v>83.35551001251559</v>
+        <v>64.63136094743892</v>
       </c>
       <c r="T92" t="n">
-        <v>83.35551001251559</v>
+        <v>64.63136094743892</v>
       </c>
     </row>
     <row r="93">
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="S93" t="n">
-        <v>84.66431799103002</v>
+        <v>65.90223264718266</v>
       </c>
       <c r="T93" t="n">
-        <v>84.66431799103002</v>
+        <v>65.90223264718266</v>
       </c>
     </row>
     <row r="94">
@@ -7410,10 +7410,10 @@
         <v>0</v>
       </c>
       <c r="S94" t="n">
-        <v>71.27810684331047</v>
+        <v>52.9040257339419</v>
       </c>
       <c r="T94" t="n">
-        <v>71.27810684331047</v>
+        <v>52.9040257339419</v>
       </c>
     </row>
     <row r="95">
@@ -7553,13 +7553,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R96" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>85.6365669392568</v>
+        <v>63.02151883406594</v>
       </c>
       <c r="T96" t="n">
-        <v>85.6365669392568</v>
+        <v>63.02151883406594</v>
       </c>
     </row>
     <row r="97">
@@ -7627,13 +7627,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R97" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S97" t="n">
-        <v>85.05952472081626</v>
+        <v>62.46120239574027</v>
       </c>
       <c r="T97" t="n">
-        <v>85.05952472081626</v>
+        <v>62.46120239574027</v>
       </c>
     </row>
     <row r="98">
@@ -7701,13 +7701,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R98" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>84.94411627712816</v>
+        <v>62.34913910807515</v>
       </c>
       <c r="T98" t="n">
-        <v>84.94411627712816</v>
+        <v>62.34913910807515</v>
       </c>
     </row>
     <row r="99">
@@ -7775,13 +7775,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R99" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>84.82870783344005</v>
+        <v>62.23707582041001</v>
       </c>
       <c r="T99" t="n">
-        <v>84.82870783344005</v>
+        <v>62.23707582041001</v>
       </c>
     </row>
     <row r="100">
@@ -7849,13 +7849,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R100" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>80.78941230435632</v>
+        <v>58.31486075213036</v>
       </c>
       <c r="T100" t="n">
-        <v>80.78941230435632</v>
+        <v>58.31486075213036</v>
       </c>
     </row>
     <row r="101">
@@ -7923,13 +7923,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R101" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>81.98908150914407</v>
+        <v>59.47975710548952</v>
       </c>
       <c r="T101" t="n">
-        <v>81.98908150914407</v>
+        <v>59.47975710548952</v>
       </c>
     </row>
     <row r="102">
@@ -7997,13 +7997,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R102" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>75.96553222804965</v>
+        <v>53.63080260718054</v>
       </c>
       <c r="T102" t="n">
-        <v>75.96553222804965</v>
+        <v>53.63080260718054</v>
       </c>
     </row>
     <row r="103">
@@ -8071,13 +8071,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R103" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>76.17307455683205</v>
+        <v>53.83232924552504</v>
       </c>
       <c r="T103" t="n">
-        <v>76.17307455683205</v>
+        <v>53.83232924552504</v>
       </c>
     </row>
     <row r="104">
@@ -8145,13 +8145,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R104" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>53.09138581921074</v>
+        <v>31.41967171249845</v>
       </c>
       <c r="T104" t="n">
-        <v>53.09138581921074</v>
+        <v>31.41967171249845</v>
       </c>
     </row>
     <row r="105">
@@ -8219,7 +8219,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R105" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
@@ -8289,7 +8289,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R106" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr"/>
@@ -8364,10 +8364,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>84.83946956184366</v>
+        <v>71.34180273475326</v>
       </c>
       <c r="T107" t="n">
-        <v>84.83946956184366</v>
+        <v>71.34180273475326</v>
       </c>
     </row>
     <row r="108">
@@ -8438,10 +8438,10 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>79.67699746785466</v>
+        <v>66.32896678580502</v>
       </c>
       <c r="T108" t="n">
-        <v>79.67699746785466</v>
+        <v>66.32896678580502</v>
       </c>
     </row>
     <row r="109">
@@ -8512,10 +8512,10 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>79.22203265720329</v>
+        <v>65.88718929687774</v>
       </c>
       <c r="T109" t="n">
-        <v>79.22203265720329</v>
+        <v>65.88718929687774</v>
       </c>
     </row>
     <row r="110">
@@ -8586,10 +8586,10 @@
         <v>0</v>
       </c>
       <c r="S110" t="n">
-        <v>81.48479333674184</v>
+        <v>68.08436302910276</v>
       </c>
       <c r="T110" t="n">
-        <v>81.48479333674184</v>
+        <v>68.08436302910276</v>
       </c>
     </row>
     <row r="111">
@@ -8660,10 +8660,10 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>74.58139158855934</v>
+        <v>61.38105890981949</v>
       </c>
       <c r="T111" t="n">
-        <v>74.58139158855934</v>
+        <v>61.38105890981949</v>
       </c>
     </row>
     <row r="112">
@@ -8734,10 +8734,10 @@
         <v>0</v>
       </c>
       <c r="S112" t="n">
-        <v>72.30656753530249</v>
+        <v>59.17217146518308</v>
       </c>
       <c r="T112" t="n">
-        <v>72.30656753530249</v>
+        <v>59.17217146518308</v>
       </c>
     </row>
     <row r="113">
@@ -8808,10 +8808,10 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>72.03358864891166</v>
+        <v>58.90710497182672</v>
       </c>
       <c r="T113" t="n">
-        <v>72.03358864891166</v>
+        <v>58.90710497182672</v>
       </c>
     </row>
     <row r="114">
@@ -8882,10 +8882,10 @@
         <v>0</v>
       </c>
       <c r="S114" t="n">
-        <v>71.76060976252086</v>
+        <v>58.64203847847035</v>
       </c>
       <c r="T114" t="n">
-        <v>71.76060976252086</v>
+        <v>58.64203847847035</v>
       </c>
     </row>
     <row r="115">
@@ -8956,10 +8956,10 @@
         <v>0</v>
       </c>
       <c r="S115" t="n">
-        <v>68.95189131020066</v>
+        <v>55.91473175953259</v>
       </c>
       <c r="T115" t="n">
-        <v>68.95189131020066</v>
+        <v>55.91473175953259</v>
       </c>
     </row>
     <row r="116">
@@ -9030,10 +9030,10 @@
         <v>0</v>
       </c>
       <c r="S116" t="n">
-        <v>67.66592646665853</v>
+        <v>54.66604107812483</v>
       </c>
       <c r="T116" t="n">
-        <v>67.66592646665853</v>
+        <v>54.66604107812483</v>
       </c>
     </row>
     <row r="117">
@@ -9104,10 +9104,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>67.57493350452826</v>
+        <v>54.57768558033938</v>
       </c>
       <c r="T117" t="n">
-        <v>67.57493350452826</v>
+        <v>54.57768558033938</v>
       </c>
     </row>
     <row r="118">
@@ -9178,10 +9178,10 @@
         <v>0</v>
       </c>
       <c r="S118" t="n">
-        <v>61.20542615540909</v>
+        <v>48.39280073535746</v>
       </c>
       <c r="T118" t="n">
-        <v>61.20542615540909</v>
+        <v>48.39280073535746</v>
       </c>
     </row>
     <row r="119">
@@ -10208,10 +10208,10 @@
         <v>0</v>
       </c>
       <c r="S133" t="n">
-        <v>78.44045906028938</v>
+        <v>65.02480939020479</v>
       </c>
       <c r="T133" t="n">
-        <v>78.44045906028938</v>
+        <v>65.02480939020479</v>
       </c>
     </row>
     <row r="134">
@@ -10282,10 +10282,10 @@
         <v>0</v>
       </c>
       <c r="S134" t="n">
-        <v>79.45642034657226</v>
+        <v>66.01132266638277</v>
       </c>
       <c r="T134" t="n">
-        <v>79.45642034657226</v>
+        <v>66.01132266638277</v>
       </c>
     </row>
     <row r="135">
@@ -10356,10 +10356,10 @@
         <v>0</v>
       </c>
       <c r="S135" t="n">
-        <v>78.45307608003282</v>
+        <v>65.0370607010084</v>
       </c>
       <c r="T135" t="n">
-        <v>78.45307608003282</v>
+        <v>65.0370607010084</v>
       </c>
     </row>
     <row r="136">
@@ -10430,10 +10430,10 @@
         <v>0</v>
       </c>
       <c r="S136" t="n">
-        <v>78.11862799118633</v>
+        <v>64.71230671255027</v>
       </c>
       <c r="T136" t="n">
-        <v>78.11862799118633</v>
+        <v>64.71230671255027</v>
       </c>
     </row>
     <row r="137">
@@ -10504,10 +10504,10 @@
         <v>0</v>
       </c>
       <c r="S137" t="n">
-        <v>77.11528372464687</v>
+        <v>63.73804474717591</v>
       </c>
       <c r="T137" t="n">
-        <v>77.11528372464687</v>
+        <v>63.73804474717591</v>
       </c>
     </row>
     <row r="138">
@@ -10578,10 +10578,10 @@
         <v>0</v>
       </c>
       <c r="S138" t="n">
-        <v>74.42708199413158</v>
+        <v>61.1277615287073</v>
       </c>
       <c r="T138" t="n">
-        <v>74.42708199413158</v>
+        <v>61.1277615287073</v>
       </c>
     </row>
     <row r="139">
@@ -10652,10 +10652,10 @@
         <v>0</v>
       </c>
       <c r="S139" t="n">
-        <v>69.6165033610074</v>
+        <v>56.45661927973602</v>
       </c>
       <c r="T139" t="n">
-        <v>69.6165033610074</v>
+        <v>56.45661927973602</v>
       </c>
     </row>
     <row r="140">
@@ -10726,10 +10726,10 @@
         <v>0</v>
       </c>
       <c r="S140" t="n">
-        <v>70.74815301682024</v>
+        <v>57.55546765566791</v>
       </c>
       <c r="T140" t="n">
-        <v>70.74815301682024</v>
+        <v>57.55546765566791</v>
       </c>
     </row>
     <row r="141">
@@ -10800,10 +10800,10 @@
         <v>0</v>
       </c>
       <c r="S141" t="n">
-        <v>72.90123780518117</v>
+        <v>59.64614449260353</v>
       </c>
       <c r="T141" t="n">
-        <v>72.90123780518117</v>
+        <v>59.64614449260353</v>
       </c>
     </row>
     <row r="142">
@@ -10874,10 +10874,10 @@
         <v>0</v>
       </c>
       <c r="S142" t="n">
-        <v>69.55675691671632</v>
+        <v>56.39860460802227</v>
       </c>
       <c r="T142" t="n">
-        <v>69.55675691671632</v>
+        <v>56.39860460802227</v>
       </c>
     </row>
     <row r="143">
@@ -10948,10 +10948,10 @@
         <v>0</v>
       </c>
       <c r="S143" t="n">
-        <v>66.86855518620104</v>
+        <v>53.78832138955367</v>
       </c>
       <c r="T143" t="n">
-        <v>66.86855518620104</v>
+        <v>53.78832138955367</v>
       </c>
     </row>
     <row r="144">
@@ -11022,10 +11022,10 @@
         <v>0</v>
       </c>
       <c r="S144" t="n">
-        <v>63.39576890846279</v>
+        <v>50.4161950944149</v>
       </c>
       <c r="T144" t="n">
-        <v>63.39576890846279</v>
+        <v>50.4161950944149</v>
       </c>
     </row>
     <row r="145">
@@ -11096,10 +11096,10 @@
         <v>0</v>
       </c>
       <c r="S145" t="n">
-        <v>61.53000278440069</v>
+        <v>48.60450888502728</v>
       </c>
       <c r="T145" t="n">
-        <v>61.53000278440069</v>
+        <v>48.60450888502728</v>
       </c>
     </row>
     <row r="146">
@@ -11242,10 +11242,10 @@
         <v>0</v>
       </c>
       <c r="S147" t="n">
-        <v>83.41203967840545</v>
+        <v>70.00082913431056</v>
       </c>
       <c r="T147" t="n">
-        <v>83.41203967840545</v>
+        <v>70.00082913431056</v>
       </c>
     </row>
     <row r="148">
@@ -11316,10 +11316,10 @@
         <v>0</v>
       </c>
       <c r="S148" t="n">
-        <v>88.94471104206679</v>
+        <v>75.37313399146826</v>
       </c>
       <c r="T148" t="n">
-        <v>88.94471104206679</v>
+        <v>75.37313399146826</v>
       </c>
     </row>
     <row r="149">
@@ -11390,10 +11390,10 @@
         <v>0</v>
       </c>
       <c r="S149" t="n">
-        <v>85.22300688439542</v>
+        <v>71.7593047923433</v>
       </c>
       <c r="T149" t="n">
-        <v>85.22300688439542</v>
+        <v>71.7593047923433</v>
       </c>
     </row>
     <row r="150">
@@ -11464,10 +11464,10 @@
         <v>0</v>
       </c>
       <c r="S150" t="n">
-        <v>76.79379544338643</v>
+        <v>63.57441713319739</v>
       </c>
       <c r="T150" t="n">
-        <v>76.79379544338643</v>
+        <v>63.57441713319739</v>
       </c>
     </row>
     <row r="151">
@@ -11538,10 +11538,10 @@
         <v>0</v>
       </c>
       <c r="S151" t="n">
-        <v>77.19623260027309</v>
+        <v>63.96518950164911</v>
       </c>
       <c r="T151" t="n">
-        <v>77.19623260027309</v>
+        <v>63.96518950164911</v>
       </c>
     </row>
     <row r="152">
@@ -11612,10 +11612,10 @@
         <v>0</v>
       </c>
       <c r="S152" t="n">
-        <v>79.95242339882857</v>
+        <v>66.64149110011131</v>
       </c>
       <c r="T152" t="n">
-        <v>79.95242339882857</v>
+        <v>66.64149110011131</v>
       </c>
     </row>
     <row r="153">
@@ -11686,10 +11686,10 @@
         <v>0</v>
       </c>
       <c r="S153" t="n">
-        <v>71.92564911470625</v>
+        <v>58.8473758094171</v>
       </c>
       <c r="T153" t="n">
-        <v>71.92564911470625</v>
+        <v>58.8473758094171</v>
       </c>
     </row>
     <row r="154">
@@ -11760,10 +11760,10 @@
         <v>0</v>
       </c>
       <c r="S154" t="n">
-        <v>72.52930485003623</v>
+        <v>59.43353436209468</v>
       </c>
       <c r="T154" t="n">
-        <v>72.52930485003623</v>
+        <v>59.43353436209468</v>
       </c>
     </row>
     <row r="155">
@@ -11834,10 +11834,10 @@
         <v>0</v>
       </c>
       <c r="S155" t="n">
-        <v>82.54797515204149</v>
+        <v>69.16180983481421</v>
       </c>
       <c r="T155" t="n">
-        <v>82.54797515204149</v>
+        <v>69.16180983481421</v>
       </c>
     </row>
     <row r="156">
@@ -11908,10 +11908,10 @@
         <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>75.41671031078151</v>
+        <v>62.23724731768945</v>
       </c>
       <c r="T156" t="n">
-        <v>75.41671031078151</v>
+        <v>62.23724731768945</v>
       </c>
     </row>
     <row r="157">
@@ -11982,10 +11982,10 @@
         <v>0</v>
       </c>
       <c r="S157" t="n">
-        <v>79.74207020378284</v>
+        <v>66.43723506949196</v>
       </c>
       <c r="T157" t="n">
-        <v>79.74207020378284</v>
+        <v>66.43723506949196</v>
       </c>
     </row>
     <row r="158">
@@ -12056,10 +12056,10 @@
         <v>0</v>
       </c>
       <c r="S158" t="n">
-        <v>66.44471243409366</v>
+        <v>53.52530608656576</v>
       </c>
       <c r="T158" t="n">
-        <v>66.44471243409366</v>
+        <v>53.52530608656576</v>
       </c>
     </row>
     <row r="159">
@@ -12130,10 +12130,10 @@
         <v>0</v>
       </c>
       <c r="S159" t="n">
-        <v>61.95871349574973</v>
+        <v>49.16933547100392</v>
       </c>
       <c r="T159" t="n">
-        <v>61.95871349574973</v>
+        <v>49.16933547100392</v>
       </c>
     </row>
     <row r="160">
@@ -12204,10 +12204,10 @@
         <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>52.6857272949272</v>
+        <v>40.16513017259493</v>
       </c>
       <c r="T160" t="n">
-        <v>52.6857272949272</v>
+        <v>40.16513017259493</v>
       </c>
     </row>
     <row r="161">
@@ -12278,10 +12278,10 @@
         <v>0</v>
       </c>
       <c r="S161" t="n">
-        <v>48.03908931124072</v>
+        <v>35.65317669327378</v>
       </c>
       <c r="T161" t="n">
-        <v>48.03908931124072</v>
+        <v>35.65317669327378</v>
       </c>
     </row>
     <row r="162">
@@ -12352,10 +12352,10 @@
         <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>40.97782838623426</v>
+        <v>28.79658900324231</v>
       </c>
       <c r="T162" t="n">
-        <v>40.97782838623426</v>
+        <v>28.79658900324231</v>
       </c>
     </row>
     <row r="163">
@@ -12428,10 +12428,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>88.22238373317265</v>
+        <v>74.60672137376142</v>
       </c>
       <c r="T163" t="n">
-        <v>88.22238373317265</v>
+        <v>74.60672137376142</v>
       </c>
     </row>
     <row r="164">
@@ -12502,10 +12502,10 @@
         <v>0</v>
       </c>
       <c r="S164" t="n">
-        <v>81.86501536293974</v>
+        <v>68.43362365491534</v>
       </c>
       <c r="T164" t="n">
-        <v>81.86501536293974</v>
+        <v>68.43362365491534</v>
       </c>
     </row>
     <row r="165">
@@ -12576,10 +12576,10 @@
         <v>0</v>
       </c>
       <c r="S165" t="n">
-        <v>83.64191797816034</v>
+        <v>70.15902209682253</v>
       </c>
       <c r="T165" t="n">
-        <v>83.64191797816034</v>
+        <v>70.15902209682253</v>
       </c>
     </row>
     <row r="166">
@@ -12650,10 +12650,10 @@
         <v>0</v>
       </c>
       <c r="S166" t="n">
-        <v>64.99728698831352</v>
+        <v>52.0548125671278</v>
       </c>
       <c r="T166" t="n">
-        <v>64.99728698831352</v>
+        <v>52.0548125671278</v>
       </c>
     </row>
     <row r="167">
@@ -12724,10 +12724,10 @@
         <v>0</v>
       </c>
       <c r="S167" t="n">
-        <v>67.18965664508356</v>
+        <v>54.18363558616873</v>
       </c>
       <c r="T167" t="n">
-        <v>67.18965664508356</v>
+        <v>54.18363558616873</v>
       </c>
     </row>
     <row r="168">
@@ -12798,10 +12798,10 @@
         <v>0</v>
       </c>
       <c r="S168" t="n">
-        <v>73.2932777149326</v>
+        <v>60.11034096309903</v>
       </c>
       <c r="T168" t="n">
-        <v>73.2932777149326</v>
+        <v>60.11034096309903</v>
       </c>
     </row>
     <row r="169">
@@ -12872,10 +12872,10 @@
         <v>0</v>
       </c>
       <c r="S169" t="n">
-        <v>60.09438901977044</v>
+        <v>47.29402689249816</v>
       </c>
       <c r="T169" t="n">
-        <v>60.09438901977044</v>
+        <v>47.29402689249816</v>
       </c>
     </row>
     <row r="170">
@@ -13018,10 +13018,10 @@
         <v>0</v>
       </c>
       <c r="S171" t="n">
-        <v>78.7249536788154</v>
+        <v>65.29497327590074</v>
       </c>
       <c r="T171" t="n">
-        <v>78.7249536788154</v>
+        <v>65.29497327590074</v>
       </c>
     </row>
     <row r="172">
@@ -13092,10 +13092,10 @@
         <v>0</v>
       </c>
       <c r="S172" t="n">
-        <v>76.31405304180255</v>
+        <v>62.95395347714346</v>
       </c>
       <c r="T172" t="n">
-        <v>76.31405304180255</v>
+        <v>62.95395347714346</v>
       </c>
     </row>
     <row r="173">
@@ -13166,10 +13166,10 @@
         <v>0</v>
       </c>
       <c r="S173" t="n">
-        <v>75.45210155661215</v>
+        <v>62.11698597154808</v>
       </c>
       <c r="T173" t="n">
-        <v>75.45210155661215</v>
+        <v>62.11698597154808</v>
       </c>
     </row>
     <row r="174">
@@ -13240,10 +13240,10 @@
         <v>0</v>
       </c>
       <c r="S174" t="n">
-        <v>68.88969020210847</v>
+        <v>55.74478851445276</v>
       </c>
       <c r="T174" t="n">
-        <v>68.88969020210847</v>
+        <v>55.74478851445276</v>
       </c>
     </row>
     <row r="175">
@@ -13314,10 +13314,10 @@
         <v>0</v>
       </c>
       <c r="S175" t="n">
-        <v>63.24286449561298</v>
+        <v>50.26163811991117</v>
       </c>
       <c r="T175" t="n">
-        <v>63.24286449561298</v>
+        <v>50.26163811991117</v>
       </c>
     </row>
     <row r="176">
@@ -13388,10 +13388,10 @@
         <v>0</v>
       </c>
       <c r="S176" t="n">
-        <v>66.4490765124123</v>
+        <v>53.37491690673028</v>
       </c>
       <c r="T176" t="n">
-        <v>66.4490765124123</v>
+        <v>53.37491690673028</v>
       </c>
     </row>
     <row r="177">
@@ -13534,10 +13534,10 @@
         <v>0</v>
       </c>
       <c r="S178" t="n">
-        <v>69.85278724697778</v>
+        <v>50.91033753556178</v>
       </c>
       <c r="T178" t="n">
-        <v>69.85278724697778</v>
+        <v>50.91033753556178</v>
       </c>
     </row>
     <row r="179">
@@ -13608,10 +13608,10 @@
         <v>0</v>
       </c>
       <c r="S179" t="n">
-        <v>59.73932622028721</v>
+        <v>41.0900188820408</v>
       </c>
       <c r="T179" t="n">
-        <v>59.73932622028721</v>
+        <v>41.0900188820408</v>
       </c>
     </row>
     <row r="180">
@@ -13682,10 +13682,10 @@
         <v>0</v>
       </c>
       <c r="S180" t="n">
-        <v>59.10723490611905</v>
+        <v>40.47624896619574</v>
       </c>
       <c r="T180" t="n">
-        <v>59.10723490611905</v>
+        <v>40.47624896619574</v>
       </c>
     </row>
     <row r="181">
@@ -13756,10 +13756,10 @@
         <v>0</v>
       </c>
       <c r="S181" t="n">
-        <v>57.21096096361457</v>
+        <v>38.63493921866056</v>
       </c>
       <c r="T181" t="n">
-        <v>57.21096096361457</v>
+        <v>38.63493921866056</v>
       </c>
     </row>
     <row r="182">
@@ -13830,10 +13830,10 @@
         <v>0</v>
       </c>
       <c r="S182" t="n">
-        <v>53.4184130786056</v>
+        <v>34.95231972359019</v>
       </c>
       <c r="T182" t="n">
-        <v>53.4184130786056</v>
+        <v>34.95231972359019</v>
       </c>
     </row>
     <row r="183">
@@ -13904,10 +13904,10 @@
         <v>0</v>
       </c>
       <c r="S183" t="n">
-        <v>23.07802999853383</v>
+        <v>5.491363763027268</v>
       </c>
       <c r="T183" t="n">
-        <v>23.07802999853383</v>
+        <v>5.491363763027268</v>
       </c>
     </row>
     <row r="184">
@@ -13980,10 +13980,10 @@
         <v>0</v>
       </c>
       <c r="S184" t="n">
-        <v>71.47243518840469</v>
+        <v>52.48303938800922</v>
       </c>
       <c r="T184" t="n">
-        <v>71.47243518840469</v>
+        <v>52.48303938800922</v>
       </c>
     </row>
     <row r="185">
@@ -14054,10 +14054,10 @@
         <v>0</v>
       </c>
       <c r="S185" t="n">
-        <v>66.40681882798269</v>
+        <v>47.5642517737051</v>
       </c>
       <c r="T185" t="n">
-        <v>66.40681882798269</v>
+        <v>47.5642517737051</v>
       </c>
     </row>
     <row r="186">
@@ -14128,10 +14128,10 @@
         <v>0</v>
       </c>
       <c r="S186" t="n">
-        <v>61.34120246756069</v>
+        <v>42.64546415940097</v>
       </c>
       <c r="T186" t="n">
-        <v>61.34120246756069</v>
+        <v>42.64546415940097</v>
       </c>
     </row>
     <row r="187">
@@ -14202,10 +14202,10 @@
         <v>0</v>
       </c>
       <c r="S187" t="n">
-        <v>60.07479837745519</v>
+        <v>41.41576725582492</v>
       </c>
       <c r="T187" t="n">
-        <v>60.07479837745519</v>
+        <v>41.41576725582492</v>
       </c>
     </row>
     <row r="188">
@@ -14276,10 +14276,10 @@
         <v>0</v>
       </c>
       <c r="S188" t="n">
-        <v>59.44159633240243</v>
+        <v>40.8009188040369</v>
       </c>
       <c r="T188" t="n">
-        <v>59.44159633240243</v>
+        <v>40.8009188040369</v>
       </c>
     </row>
     <row r="189">
@@ -14350,10 +14350,10 @@
         <v>0</v>
       </c>
       <c r="S189" t="n">
-        <v>53.10957588187494</v>
+        <v>34.65243428615675</v>
       </c>
       <c r="T189" t="n">
-        <v>53.10957588187494</v>
+        <v>34.65243428615675</v>
       </c>
     </row>
     <row r="190">
@@ -14424,10 +14424,10 @@
         <v>0</v>
       </c>
       <c r="S190" t="n">
-        <v>42.37281315235018</v>
+        <v>24.2268805580199</v>
       </c>
       <c r="T190" t="n">
-        <v>42.37281315235018</v>
+        <v>24.2268805580199</v>
       </c>
     </row>
     <row r="191">
@@ -14500,10 +14500,10 @@
         <v>0</v>
       </c>
       <c r="S191" t="n">
-        <v>54.19893031982607</v>
+        <v>35.71021338661252</v>
       </c>
       <c r="T191" t="n">
-        <v>54.19893031982607</v>
+        <v>35.71021338661252</v>
       </c>
     </row>
     <row r="192">
@@ -14574,10 +14574,10 @@
         <v>0</v>
       </c>
       <c r="S192" t="n">
-        <v>54.81189755523987</v>
+        <v>36.30541354213249</v>
       </c>
       <c r="T192" t="n">
-        <v>54.81189755523987</v>
+        <v>36.30541354213249</v>
       </c>
     </row>
     <row r="193">
@@ -14648,10 +14648,10 @@
         <v>0</v>
       </c>
       <c r="S193" t="n">
-        <v>59.42500968620467</v>
+        <v>40.78481292785611</v>
       </c>
       <c r="T193" t="n">
-        <v>59.42500968620467</v>
+        <v>40.78481292785611</v>
       </c>
     </row>
     <row r="194">
@@ -14722,10 +14722,10 @@
         <v>0</v>
       </c>
       <c r="S194" t="n">
-        <v>60.52220301878641</v>
+        <v>41.85020370970965</v>
       </c>
       <c r="T194" t="n">
-        <v>60.52220301878641</v>
+        <v>41.85020370970965</v>
       </c>
     </row>
     <row r="195">
@@ -14796,10 +14796,10 @@
         <v>0</v>
       </c>
       <c r="S195" t="n">
-        <v>43.4145847887352</v>
+        <v>25.23845606184607</v>
       </c>
       <c r="T195" t="n">
-        <v>43.4145847887352</v>
+        <v>25.23845606184607</v>
       </c>
     </row>
     <row r="196">
@@ -14870,10 +14870,10 @@
         <v>0</v>
       </c>
       <c r="S196" t="n">
-        <v>42.15189931199622</v>
+        <v>24.01236998626573</v>
       </c>
       <c r="T196" t="n">
-        <v>42.15189931199622</v>
+        <v>24.01236998626573</v>
       </c>
     </row>
     <row r="197">
@@ -14944,10 +14944,10 @@
         <v>0</v>
       </c>
       <c r="S197" t="n">
-        <v>47.48462416605144</v>
+        <v>29.19052385665346</v>
       </c>
       <c r="T197" t="n">
-        <v>47.48462416605144</v>
+        <v>29.19052385665346</v>
       </c>
     </row>
     <row r="198">
@@ -15018,10 +15018,10 @@
         <v>0</v>
       </c>
       <c r="S198" t="n">
-        <v>36.15720588131201</v>
+        <v>18.19143494097079</v>
       </c>
       <c r="T198" t="n">
-        <v>36.15720588131201</v>
+        <v>18.19143494097079</v>
       </c>
     </row>
     <row r="199">
@@ -15092,10 +15092,10 @@
         <v>0</v>
       </c>
       <c r="S199" t="n">
-        <v>14.16433788846213</v>
+        <v>-3.163961715487376</v>
       </c>
       <c r="T199" t="n">
-        <v>14.16433788846213</v>
+        <v>-3.163961715487376</v>
       </c>
     </row>
     <row r="200">
@@ -15166,10 +15166,10 @@
         <v>0</v>
       </c>
       <c r="S200" t="n">
-        <v>18.39986940993562</v>
+        <v>0.9488013730468206</v>
       </c>
       <c r="T200" t="n">
-        <v>18.39986940993562</v>
+        <v>0.9488013730468206</v>
       </c>
     </row>
     <row r="201">
@@ -15312,10 +15312,10 @@
         <v>0</v>
       </c>
       <c r="S202" t="n">
-        <v>68.31220950831225</v>
+        <v>52.89416515612406</v>
       </c>
       <c r="T202" t="n">
-        <v>68.31220950831225</v>
+        <v>52.89416515612406</v>
       </c>
     </row>
     <row r="203">
@@ -15386,10 +15386,10 @@
         <v>0</v>
       </c>
       <c r="S203" t="n">
-        <v>67.71029126490714</v>
+        <v>52.30969373353135</v>
       </c>
       <c r="T203" t="n">
-        <v>67.71029126490714</v>
+        <v>52.30969373353135</v>
       </c>
     </row>
     <row r="204">
@@ -15460,10 +15460,10 @@
         <v>0</v>
       </c>
       <c r="S204" t="n">
-        <v>72.18121291247532</v>
+        <v>56.65102407911452</v>
       </c>
       <c r="T204" t="n">
-        <v>72.18121291247532</v>
+        <v>56.65102407911452</v>
       </c>
     </row>
     <row r="205">
@@ -15534,10 +15534,10 @@
         <v>0</v>
       </c>
       <c r="S205" t="n">
-        <v>64.70070004788161</v>
+        <v>49.38733662056782</v>
       </c>
       <c r="T205" t="n">
-        <v>64.70070004788161</v>
+        <v>49.38733662056782</v>
       </c>
     </row>
     <row r="206">
@@ -15608,10 +15608,10 @@
         <v>0</v>
       </c>
       <c r="S206" t="n">
-        <v>62.29302707426118</v>
+        <v>47.04945093019699</v>
       </c>
       <c r="T206" t="n">
-        <v>62.29302707426118</v>
+        <v>47.04945093019699</v>
       </c>
     </row>
     <row r="207">
@@ -15682,10 +15682,10 @@
         <v>0</v>
       </c>
       <c r="S207" t="n">
-        <v>60.48727234404585</v>
+        <v>45.29603666241886</v>
       </c>
       <c r="T207" t="n">
-        <v>60.48727234404585</v>
+        <v>45.29603666241886</v>
       </c>
     </row>
     <row r="208">
@@ -15756,10 +15756,10 @@
         <v>0</v>
       </c>
       <c r="S208" t="n">
-        <v>66.52318142446732</v>
+        <v>51.15699270674308</v>
       </c>
       <c r="T208" t="n">
-        <v>66.52318142446732</v>
+        <v>51.15699270674308</v>
       </c>
     </row>
     <row r="209">
@@ -15829,13 +15829,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R209" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S209" t="n">
-        <v>85.10868710825123</v>
+        <v>60.21905863934744</v>
       </c>
       <c r="T209" t="n">
-        <v>85.10868710825123</v>
+        <v>60.21905863934744</v>
       </c>
     </row>
     <row r="210">
@@ -15903,13 +15903,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R210" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S210" t="n">
-        <v>80.63711930114985</v>
+        <v>55.87710086340189</v>
       </c>
       <c r="T210" t="n">
-        <v>80.63711930114985</v>
+        <v>55.87710086340189</v>
       </c>
     </row>
     <row r="211">
@@ -15977,13 +15977,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R211" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S211" t="n">
-        <v>80.07817332526218</v>
+        <v>55.33435614140869</v>
       </c>
       <c r="T211" t="n">
-        <v>80.07817332526218</v>
+        <v>55.33435614140869</v>
       </c>
     </row>
     <row r="212">
@@ -16051,13 +16051,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R212" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S212" t="n">
-        <v>78.40133539759915</v>
+        <v>53.7061219754291</v>
       </c>
       <c r="T212" t="n">
-        <v>78.40133539759915</v>
+        <v>53.7061219754291</v>
       </c>
     </row>
     <row r="213">
@@ -16125,13 +16125,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R213" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S213" t="n">
-        <v>77.84238942171149</v>
+        <v>53.1633772534359</v>
       </c>
       <c r="T213" t="n">
-        <v>77.84238942171149</v>
+        <v>53.1633772534359</v>
       </c>
     </row>
     <row r="214">
@@ -16199,13 +16199,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R214" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S214" t="n">
-        <v>64.87896314307788</v>
+        <v>40.57570063495316</v>
       </c>
       <c r="T214" t="n">
-        <v>64.87896314307788</v>
+        <v>40.57570063495316</v>
       </c>
     </row>
     <row r="215">
@@ -16273,13 +16273,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R215" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S215" t="n">
-        <v>56.60244233797994</v>
+        <v>32.5390778176945</v>
       </c>
       <c r="T215" t="n">
-        <v>56.60244233797994</v>
+        <v>32.5390778176945</v>
       </c>
     </row>
     <row r="216">
@@ -16347,13 +16347,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R216" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S216" t="n">
-        <v>56.04349636209226</v>
+        <v>31.99633309570131</v>
       </c>
       <c r="T216" t="n">
-        <v>56.04349636209226</v>
+        <v>31.99633309570131</v>
       </c>
     </row>
     <row r="217">
@@ -16421,13 +16421,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R217" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S217" t="n">
-        <v>52.68982050676622</v>
+        <v>28.73986476374214</v>
       </c>
       <c r="T217" t="n">
-        <v>52.68982050676622</v>
+        <v>28.73986476374214</v>
       </c>
     </row>
     <row r="218">
@@ -16495,13 +16495,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R218" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S218" t="n">
-        <v>52.46624211641115</v>
+        <v>28.52276687494486</v>
       </c>
       <c r="T218" t="n">
-        <v>52.46624211641115</v>
+        <v>28.52276687494486</v>
       </c>
     </row>
     <row r="219">
@@ -16569,7 +16569,7 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R219" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S219" t="inlineStr"/>
       <c r="T219" t="inlineStr"/>
@@ -16644,10 +16644,10 @@
         <v>0</v>
       </c>
       <c r="S220" t="n">
-        <v>88.91858090053606</v>
+        <v>73.21879496443654</v>
       </c>
       <c r="T220" t="n">
-        <v>88.91858090053606</v>
+        <v>73.21879496443654</v>
       </c>
     </row>
     <row r="221">
@@ -16718,10 +16718,10 @@
         <v>0</v>
       </c>
       <c r="S221" t="n">
-        <v>76.97474437915585</v>
+        <v>61.62115492054184</v>
       </c>
       <c r="T221" t="n">
-        <v>76.97474437915585</v>
+        <v>61.62115492054184</v>
       </c>
     </row>
     <row r="222">
@@ -16792,10 +16792,10 @@
         <v>0</v>
       </c>
       <c r="S222" t="n">
-        <v>74.32401917761355</v>
+        <v>59.04726196012352</v>
       </c>
       <c r="T222" t="n">
-        <v>74.32401917761355</v>
+        <v>59.04726196012352</v>
       </c>
     </row>
     <row r="223">
@@ -16866,10 +16866,10 @@
         <v>0</v>
       </c>
       <c r="S223" t="n">
-        <v>69.73841514111328</v>
+        <v>54.59457333666813</v>
       </c>
       <c r="T223" t="n">
-        <v>69.73841514111328</v>
+        <v>54.59457333666813</v>
       </c>
     </row>
     <row r="224">
@@ -16940,10 +16940,10 @@
         <v>0</v>
       </c>
       <c r="S224" t="n">
-        <v>65.99834727525463</v>
+        <v>50.9629127081657</v>
       </c>
       <c r="T224" t="n">
-        <v>65.99834727525463</v>
+        <v>50.9629127081657</v>
       </c>
     </row>
     <row r="225">
@@ -17014,10 +17014,10 @@
         <v>0</v>
       </c>
       <c r="S225" t="n">
-        <v>73.24246307051713</v>
+        <v>57.99705515304553</v>
       </c>
       <c r="T225" t="n">
-        <v>73.24246307051713</v>
+        <v>57.99705515304553</v>
       </c>
     </row>
     <row r="226">
@@ -17088,10 +17088,10 @@
         <v>0</v>
       </c>
       <c r="S226" t="n">
-        <v>64.19315824435397</v>
+        <v>49.21004774270033</v>
       </c>
       <c r="T226" t="n">
-        <v>64.19315824435397</v>
+        <v>49.21004774270033</v>
       </c>
     </row>
     <row r="227">
@@ -17162,10 +17162,10 @@
         <v>0</v>
       </c>
       <c r="S227" t="n">
-        <v>62.98969889042018</v>
+        <v>48.04147109905674</v>
       </c>
       <c r="T227" t="n">
-        <v>62.98969889042018</v>
+        <v>48.04147109905674</v>
       </c>
     </row>
     <row r="228">
@@ -17236,10 +17236,10 @@
         <v>0</v>
       </c>
       <c r="S228" t="n">
-        <v>39.22392909449714</v>
+        <v>24.96456084783295</v>
       </c>
       <c r="T228" t="n">
-        <v>39.22392909449714</v>
+        <v>24.96456084783295</v>
       </c>
     </row>
     <row r="229">
@@ -17312,10 +17312,10 @@
         <v>0</v>
       </c>
       <c r="S229" t="n">
-        <v>86.25024811922027</v>
+        <v>67.84277091512082</v>
       </c>
       <c r="T229" t="n">
-        <v>86.25024811922027</v>
+        <v>67.84277091512082</v>
       </c>
     </row>
     <row r="230">
@@ -17386,10 +17386,10 @@
         <v>0</v>
       </c>
       <c r="S230" t="n">
-        <v>79.44924041831982</v>
+        <v>61.23889291414459</v>
       </c>
       <c r="T230" t="n">
-        <v>79.44924041831982</v>
+        <v>61.23889291414459</v>
       </c>
     </row>
     <row r="231">
@@ -17460,10 +17460,10 @@
         <v>0</v>
       </c>
       <c r="S231" t="n">
-        <v>86.16158460706581</v>
+        <v>67.75667734735018</v>
       </c>
       <c r="T231" t="n">
-        <v>86.16158460706581</v>
+        <v>67.75667734735018</v>
       </c>
     </row>
     <row r="232">
@@ -17534,10 +17534,10 @@
         <v>0</v>
       </c>
       <c r="S232" t="n">
-        <v>76.61548720961129</v>
+        <v>58.48727708040449</v>
       </c>
       <c r="T232" t="n">
-        <v>76.61548720961129</v>
+        <v>58.48727708040449</v>
       </c>
     </row>
     <row r="233">
@@ -17608,10 +17608,10 @@
         <v>0</v>
       </c>
       <c r="S233" t="n">
-        <v>82.3254129456531</v>
+        <v>64.03169852701777</v>
       </c>
       <c r="T233" t="n">
-        <v>82.3254129456531</v>
+        <v>64.03169852701777</v>
       </c>
     </row>
     <row r="234">
@@ -17682,10 +17682,10 @@
         <v>0</v>
       </c>
       <c r="S234" t="n">
-        <v>66.37155633963584</v>
+        <v>48.54027029980705</v>
       </c>
       <c r="T234" t="n">
-        <v>66.37155633963584</v>
+        <v>48.54027029980705</v>
       </c>
     </row>
     <row r="235">
@@ -17756,10 +17756,10 @@
         <v>0</v>
       </c>
       <c r="S235" t="n">
-        <v>75.96007305571511</v>
+        <v>57.85086034588581</v>
       </c>
       <c r="T235" t="n">
-        <v>75.96007305571511</v>
+        <v>57.85086034588581</v>
       </c>
     </row>
     <row r="236">
@@ -17902,10 +17902,10 @@
         <v>0</v>
       </c>
       <c r="S237" t="n">
-        <v>85.86664877361795</v>
+        <v>67.39724822488002</v>
       </c>
       <c r="T237" t="n">
-        <v>85.86664877361795</v>
+        <v>67.39724822488002</v>
       </c>
     </row>
     <row r="238">
@@ -17976,10 +17976,10 @@
         <v>0</v>
       </c>
       <c r="S238" t="n">
-        <v>84.32271852797888</v>
+        <v>65.89806936306695</v>
       </c>
       <c r="T238" t="n">
-        <v>84.32271852797888</v>
+        <v>65.89806936306695</v>
       </c>
     </row>
     <row r="239">
@@ -18050,10 +18050,10 @@
         <v>0</v>
       </c>
       <c r="S239" t="n">
-        <v>56.53197410647541</v>
+        <v>38.91284985043195</v>
       </c>
       <c r="T239" t="n">
-        <v>56.53197410647541</v>
+        <v>38.91284985043195</v>
       </c>
     </row>
     <row r="240">
@@ -18124,10 +18124,10 @@
         <v>0</v>
       </c>
       <c r="S240" t="n">
-        <v>55.76000898365587</v>
+        <v>38.16326041952543</v>
       </c>
       <c r="T240" t="n">
-        <v>55.76000898365587</v>
+        <v>38.16326041952543</v>
       </c>
     </row>
     <row r="241">
@@ -18198,10 +18198,10 @@
         <v>0</v>
       </c>
       <c r="S241" t="n">
-        <v>52.67214849237771</v>
+        <v>35.16490269589931</v>
       </c>
       <c r="T241" t="n">
-        <v>52.67214849237771</v>
+        <v>35.16490269589931</v>
       </c>
     </row>
     <row r="242">
@@ -18272,10 +18272,10 @@
         <v>0</v>
       </c>
       <c r="S242" t="n">
-        <v>52.36336244324989</v>
+        <v>34.8650669235367</v>
       </c>
       <c r="T242" t="n">
-        <v>52.36336244324989</v>
+        <v>34.8650669235367</v>
       </c>
     </row>
     <row r="243">
@@ -18346,10 +18346,10 @@
         <v>0</v>
       </c>
       <c r="S243" t="n">
-        <v>45.77790001633856</v>
+        <v>28.47048653781279</v>
       </c>
       <c r="T243" t="n">
-        <v>45.77790001633856</v>
+        <v>28.47048653781279</v>
       </c>
     </row>
     <row r="244">
@@ -18420,10 +18420,10 @@
         <v>0</v>
       </c>
       <c r="S244" t="n">
-        <v>42.79099492028758</v>
+        <v>25.57015798029576</v>
       </c>
       <c r="T244" t="n">
-        <v>42.79099492028758</v>
+        <v>25.57015798029576</v>
       </c>
     </row>
     <row r="245">
@@ -18494,10 +18494,10 @@
         <v>0</v>
       </c>
       <c r="S245" t="n">
-        <v>40.47509955182896</v>
+        <v>23.32138968757617</v>
       </c>
       <c r="T245" t="n">
-        <v>40.47509955182896</v>
+        <v>23.32138968757617</v>
       </c>
     </row>
     <row r="246">
@@ -18568,10 +18568,10 @@
         <v>0</v>
       </c>
       <c r="S246" t="n">
-        <v>35.02086599447859</v>
+        <v>18.02524908817594</v>
       </c>
       <c r="T246" t="n">
-        <v>35.02086599447859</v>
+        <v>18.02524908817594</v>
       </c>
     </row>
     <row r="247">
@@ -18642,10 +18642,10 @@
         <v>0</v>
       </c>
       <c r="S247" t="n">
-        <v>27.25073706866957</v>
+        <v>10.48034019605612</v>
       </c>
       <c r="T247" t="n">
-        <v>27.25073706866957</v>
+        <v>10.48034019605612</v>
       </c>
     </row>
     <row r="248">
@@ -18716,10 +18716,10 @@
         <v>0</v>
       </c>
       <c r="S248" t="n">
-        <v>32.75544832363356</v>
+        <v>15.8254953785109</v>
       </c>
       <c r="T248" t="n">
-        <v>32.75544832363356</v>
+        <v>15.8254953785109</v>
       </c>
     </row>
     <row r="249">
@@ -18790,10 +18790,10 @@
         <v>0</v>
       </c>
       <c r="S249" t="n">
-        <v>30.43955295517492</v>
+        <v>13.57672708579131</v>
       </c>
       <c r="T249" t="n">
-        <v>30.43955295517492</v>
+        <v>13.57672708579131</v>
       </c>
     </row>
     <row r="250">
@@ -18866,10 +18866,10 @@
         <v>0</v>
       </c>
       <c r="S250" t="n">
-        <v>73.29018399548812</v>
+        <v>57.72785122898782</v>
       </c>
       <c r="T250" t="n">
-        <v>73.29018399548812</v>
+        <v>57.72785122898782</v>
       </c>
     </row>
     <row r="251">
@@ -18940,10 +18940,10 @@
         <v>0</v>
       </c>
       <c r="S251" t="n">
-        <v>69.44994028355774</v>
+        <v>53.99891838801388</v>
       </c>
       <c r="T251" t="n">
-        <v>69.44994028355774</v>
+        <v>53.99891838801388</v>
       </c>
     </row>
     <row r="252">
@@ -19014,10 +19014,10 @@
         <v>0</v>
       </c>
       <c r="S252" t="n">
-        <v>63.66933805088006</v>
+        <v>48.38586902891377</v>
       </c>
       <c r="T252" t="n">
-        <v>63.66933805088006</v>
+        <v>48.38586902891377</v>
       </c>
     </row>
     <row r="253">
@@ -19088,10 +19088,10 @@
         <v>0</v>
       </c>
       <c r="S253" t="n">
-        <v>64.95774493611049</v>
+        <v>49.63693096853677</v>
       </c>
       <c r="T253" t="n">
-        <v>64.95774493611049</v>
+        <v>49.63693096853677</v>
       </c>
     </row>
     <row r="254">
@@ -19162,10 +19162,10 @@
         <v>0</v>
       </c>
       <c r="S254" t="n">
-        <v>63.88464998677044</v>
+        <v>48.59494006945764</v>
       </c>
       <c r="T254" t="n">
-        <v>63.88464998677044</v>
+        <v>48.59494006945764</v>
       </c>
     </row>
     <row r="255">
@@ -19236,10 +19236,10 @@
         <v>0</v>
       </c>
       <c r="S255" t="n">
-        <v>61.61357536928594</v>
+        <v>46.38969338182402</v>
       </c>
       <c r="T255" t="n">
-        <v>61.61357536928594</v>
+        <v>46.38969338182402</v>
       </c>
     </row>
     <row r="256">
@@ -19310,10 +19310,10 @@
         <v>0</v>
       </c>
       <c r="S256" t="n">
-        <v>59.34250075180142</v>
+        <v>44.18444669419039</v>
       </c>
       <c r="T256" t="n">
-        <v>59.34250075180142</v>
+        <v>44.18444669419039</v>
       </c>
     </row>
     <row r="257">
@@ -19384,10 +19384,10 @@
         <v>0</v>
       </c>
       <c r="S257" t="n">
-        <v>55.66761508823965</v>
+        <v>40.61607893797018</v>
       </c>
       <c r="T257" t="n">
-        <v>55.66761508823965</v>
+        <v>40.61607893797018</v>
       </c>
     </row>
     <row r="258">
@@ -19458,10 +19458,10 @@
         <v>0</v>
       </c>
       <c r="S258" t="n">
-        <v>58.26940580246139</v>
+        <v>43.14245579511125</v>
       </c>
       <c r="T258" t="n">
-        <v>58.26940580246139</v>
+        <v>43.14245579511125</v>
       </c>
     </row>
     <row r="259">
@@ -19532,10 +19532,10 @@
         <v>0</v>
       </c>
       <c r="S259" t="n">
-        <v>52.85999299608512</v>
+        <v>37.88983680079699</v>
       </c>
       <c r="T259" t="n">
-        <v>52.85999299608512</v>
+        <v>37.88983680079699</v>
       </c>
     </row>
     <row r="260">
@@ -19606,10 +19606,10 @@
         <v>0</v>
       </c>
       <c r="S260" t="n">
-        <v>52.15808747304649</v>
+        <v>37.2082762665037</v>
       </c>
       <c r="T260" t="n">
-        <v>52.15808747304649</v>
+        <v>37.2082762665037</v>
       </c>
     </row>
     <row r="261">
@@ -19752,10 +19752,10 @@
         <v>0</v>
       </c>
       <c r="S262" t="n">
-        <v>87.13041511408375</v>
+        <v>68.90490182273359</v>
       </c>
       <c r="T262" t="n">
-        <v>87.13041511408375</v>
+        <v>68.90490182273359</v>
       </c>
     </row>
     <row r="263">
@@ -19826,10 +19826,10 @@
         <v>0</v>
       </c>
       <c r="S263" t="n">
-        <v>83.31805840299052</v>
+        <v>65.20304766766047</v>
       </c>
       <c r="T263" t="n">
-        <v>83.31805840299052</v>
+        <v>65.20304766766047</v>
       </c>
     </row>
     <row r="264">
@@ -19900,10 +19900,10 @@
         <v>0</v>
       </c>
       <c r="S264" t="n">
-        <v>87.34092479205398</v>
+        <v>69.10930980056257</v>
       </c>
       <c r="T264" t="n">
-        <v>87.34092479205398</v>
+        <v>69.10930980056257</v>
       </c>
     </row>
     <row r="265">
@@ -19974,10 +19974,10 @@
         <v>0</v>
       </c>
       <c r="S265" t="n">
-        <v>91.77882466651103</v>
+        <v>73.41857552122654</v>
       </c>
       <c r="T265" t="n">
-        <v>91.77882466651103</v>
+        <v>73.41857552122654</v>
       </c>
     </row>
     <row r="266">
@@ -20048,10 +20048,10 @@
         <v>0</v>
       </c>
       <c r="S266" t="n">
-        <v>78.77258543878546</v>
+        <v>60.78932690266683</v>
       </c>
       <c r="T266" t="n">
-        <v>78.77258543878546</v>
+        <v>60.78932690266683</v>
       </c>
     </row>
     <row r="267">
@@ -20122,10 +20122,10 @@
         <v>0</v>
       </c>
       <c r="S267" t="n">
-        <v>86.34882350213425</v>
+        <v>68.14596493001144</v>
       </c>
       <c r="T267" t="n">
-        <v>86.34882350213425</v>
+        <v>68.14596493001144</v>
       </c>
     </row>
     <row r="268">
@@ -20196,10 +20196,10 @@
         <v>0</v>
       </c>
       <c r="S268" t="n">
-        <v>84.37524329436751</v>
+        <v>66.22958966763565</v>
       </c>
       <c r="T268" t="n">
-        <v>84.37524329436751</v>
+        <v>66.22958966763565</v>
       </c>
     </row>
     <row r="269">
@@ -20270,10 +20270,10 @@
         <v>0</v>
       </c>
       <c r="S269" t="n">
-        <v>75.84475692786395</v>
+        <v>57.94636257381514</v>
       </c>
       <c r="T269" t="n">
-        <v>75.84475692786395</v>
+        <v>57.94636257381514</v>
       </c>
     </row>
     <row r="270">
@@ -20344,10 +20344,10 @@
         <v>0</v>
       </c>
       <c r="S270" t="n">
-        <v>73.82270136125953</v>
+        <v>55.9829170286377</v>
       </c>
       <c r="T270" t="n">
-        <v>73.82270136125953</v>
+        <v>55.9829170286377</v>
       </c>
     </row>
     <row r="271">
@@ -20418,10 +20418,10 @@
         <v>0</v>
       </c>
       <c r="S271" t="n">
-        <v>66.86138408920186</v>
+        <v>49.22337608815752</v>
       </c>
       <c r="T271" t="n">
-        <v>66.86138408920186</v>
+        <v>49.22337608815752</v>
       </c>
     </row>
     <row r="272">
@@ -20492,10 +20492,10 @@
         <v>0</v>
       </c>
       <c r="S272" t="n">
-        <v>68.16094577476716</v>
+        <v>50.48526950214086</v>
       </c>
       <c r="T272" t="n">
-        <v>68.16094577476716</v>
+        <v>50.48526950214086</v>
       </c>
     </row>
     <row r="273">
@@ -20566,10 +20566,10 @@
         <v>0</v>
       </c>
       <c r="S273" t="n">
-        <v>59.18819530817775</v>
+        <v>41.77259749520962</v>
       </c>
       <c r="T273" t="n">
-        <v>59.18819530817775</v>
+        <v>41.77259749520962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>